<commit_message>
updated lstm to only train once when test data is corrupted
</commit_message>
<xml_diff>
--- a/Sensor_Corruption.xlsx
+++ b/Sensor_Corruption.xlsx
@@ -409,10 +409,10 @@
         <v>0.542</v>
       </c>
       <c r="H3" s="2">
-        <v>0.9101</v>
+        <v>0.8935</v>
       </c>
       <c r="I3" s="2">
-        <v>0.9108</v>
+        <v>0.8945</v>
       </c>
     </row>
     <row r="4">
@@ -591,16 +591,16 @@
         <v>0.5421</v>
       </c>
       <c r="N4" s="2">
-        <v>0.9046</v>
+        <v>0.8938</v>
       </c>
       <c r="O4" s="2">
-        <v>0.9057</v>
+        <v>0.8949</v>
       </c>
       <c r="P4" s="2">
-        <v>0.907</v>
+        <v>0.8904</v>
       </c>
       <c r="Q4" s="2">
-        <v>0.9081</v>
+        <v>0.8913</v>
       </c>
     </row>
     <row r="5">
@@ -644,16 +644,16 @@
         <v>0.5309</v>
       </c>
       <c r="N5" s="2">
-        <v>0.906</v>
+        <v>0.8914</v>
       </c>
       <c r="O5" s="2">
-        <v>0.9068</v>
+        <v>0.8928</v>
       </c>
       <c r="P5" s="2">
-        <v>0.9046</v>
+        <v>0.889</v>
       </c>
       <c r="Q5" s="2">
-        <v>0.9045</v>
+        <v>0.8899</v>
       </c>
     </row>
     <row r="6">
@@ -697,16 +697,16 @@
         <v>0.5402</v>
       </c>
       <c r="N6" s="2">
-        <v>0.9233</v>
+        <v>0.8935</v>
       </c>
       <c r="O6" s="2">
-        <v>0.9243</v>
+        <v>0.895</v>
       </c>
       <c r="P6" s="2">
-        <v>0.889</v>
+        <v>0.8812</v>
       </c>
       <c r="Q6" s="2">
-        <v>0.8895</v>
+        <v>0.8813</v>
       </c>
     </row>
     <row r="7">
@@ -750,16 +750,16 @@
         <v>0.5268</v>
       </c>
       <c r="N7" s="2">
-        <v>0.9175</v>
+        <v>0.8785</v>
       </c>
       <c r="O7" s="2">
-        <v>0.9186</v>
+        <v>0.8801</v>
       </c>
       <c r="P7" s="2">
-        <v>0.908</v>
+        <v>0.8531</v>
       </c>
       <c r="Q7" s="2">
-        <v>0.9096</v>
+        <v>0.8487</v>
       </c>
     </row>
   </sheetData>
@@ -923,16 +923,16 @@
         <v>0.474</v>
       </c>
       <c r="N4" s="2">
-        <v>0.8616</v>
+        <v>0.8846</v>
       </c>
       <c r="O4" s="2">
-        <v>0.8639</v>
+        <v>0.8857</v>
       </c>
       <c r="P4" s="2">
-        <v>0.5948</v>
+        <v>0.886</v>
       </c>
       <c r="Q4" s="2">
-        <v>0.5626</v>
+        <v>0.8873</v>
       </c>
     </row>
     <row r="5">
@@ -976,16 +976,16 @@
         <v>0.4317</v>
       </c>
       <c r="N5" s="2">
-        <v>0.5219</v>
+        <v>0.7533</v>
       </c>
       <c r="O5" s="2">
-        <v>0.4518</v>
+        <v>0.7485</v>
       </c>
       <c r="P5" s="2">
-        <v>0.5039</v>
+        <v>0.8541</v>
       </c>
       <c r="Q5" s="2">
-        <v>0.4174</v>
+        <v>0.8547</v>
       </c>
     </row>
     <row r="6">
@@ -1029,16 +1029,16 @@
         <v>0.3495</v>
       </c>
       <c r="N6" s="2">
-        <v>0.4659</v>
+        <v>0.6145</v>
       </c>
       <c r="O6" s="2">
-        <v>0.3477</v>
+        <v>0.5463</v>
       </c>
       <c r="P6" s="2">
-        <v>0.4649</v>
+        <v>0.7112</v>
       </c>
       <c r="Q6" s="2">
-        <v>0.3497</v>
+        <v>0.6796</v>
       </c>
     </row>
     <row r="7">
@@ -1082,16 +1082,16 @@
         <v>0.2999</v>
       </c>
       <c r="N7" s="2">
-        <v>0.4567</v>
+        <v>0.6138</v>
       </c>
       <c r="O7" s="2">
-        <v>0.3243</v>
+        <v>0.5573</v>
       </c>
       <c r="P7" s="2">
-        <v>0.4628</v>
+        <v>0.5918</v>
       </c>
       <c r="Q7" s="2">
-        <v>0.3454</v>
+        <v>0.5352</v>
       </c>
     </row>
   </sheetData>
@@ -1255,20 +1255,16 @@
         <v>0.5447</v>
       </c>
       <c r="N4" s="2">
-        <f>0.9002</f>
-        <v>0.9002</v>
+        <v>0.8907</v>
       </c>
       <c r="O4" s="2">
-        <f>0.9014</f>
-        <v>0.9014</v>
+        <v>0.8917</v>
       </c>
       <c r="P4" s="2">
-        <f>0.9057</f>
-        <v>0.9057</v>
+        <v>0.8931</v>
       </c>
       <c r="Q4" s="2">
-        <f>0.9071</f>
-        <v>0.9071</v>
+        <v>0.8942</v>
       </c>
     </row>
     <row r="5">
@@ -1312,20 +1308,16 @@
         <v>0.5287</v>
       </c>
       <c r="N5" s="2">
-        <f>0.9169</f>
-        <v>0.9169</v>
+        <v>0.889</v>
       </c>
       <c r="O5" s="2">
-        <f>0.9184</f>
-        <v>0.9184</v>
+        <v>0.8897</v>
       </c>
       <c r="P5" s="2">
-        <f>0.9135</f>
-        <v>0.9135</v>
+        <v>0.8921</v>
       </c>
       <c r="Q5" s="2">
-        <f>0.9143</f>
-        <v>0.9143</v>
+        <v>0.8931</v>
       </c>
     </row>
     <row r="6">
@@ -1369,20 +1361,16 @@
         <v>0.5228</v>
       </c>
       <c r="N6" s="2">
-        <f>0.8897</f>
-        <v>0.8897</v>
+        <v>0.8819</v>
       </c>
       <c r="O6" s="2">
-        <f>0.8919</f>
-        <v>0.8919</v>
+        <v>0.8819</v>
       </c>
       <c r="P6" s="2">
-        <f>0.9253</f>
-        <v>0.9253</v>
+        <v>0.889</v>
       </c>
       <c r="Q6" s="2">
-        <f>0.9275</f>
-        <v>0.9275</v>
+        <v>0.8899</v>
       </c>
     </row>
     <row r="7">
@@ -1426,20 +1414,16 @@
         <v>0.5145</v>
       </c>
       <c r="N7" s="2">
-        <f>0.903</f>
-        <v>0.903</v>
+        <v>0.8738</v>
       </c>
       <c r="O7" s="2">
-        <f>0.9044</f>
-        <v>0.9044</v>
+        <v>0.8732</v>
       </c>
       <c r="P7" s="2">
-        <f>0.9141</f>
-        <v>0.9141</v>
+        <v>0.885</v>
       </c>
       <c r="Q7" s="2">
-        <f>0.9158</f>
-        <v>0.9158</v>
+        <v>0.8855</v>
       </c>
     </row>
   </sheetData>
@@ -1603,20 +1587,16 @@
         <v>0.4868</v>
       </c>
       <c r="N4" s="2">
-        <f>0.8873</f>
-        <v>0.8873</v>
+        <v>0.8945</v>
       </c>
       <c r="O4" s="2">
-        <f>0.8899</f>
-        <v>0.8899</v>
+        <v>0.8957</v>
       </c>
       <c r="P4" s="2">
-        <f>0.8734</f>
-        <v>0.8734</v>
+        <v>0.888</v>
       </c>
       <c r="Q4" s="2">
-        <f>0.875</f>
-        <v>0.875</v>
+        <v>0.8894</v>
       </c>
     </row>
     <row r="5">
@@ -1660,20 +1640,16 @@
         <v>0.4627</v>
       </c>
       <c r="N5" s="2">
-        <f>0.6033</f>
-        <v>0.6033</v>
+        <v>0.8592</v>
       </c>
       <c r="O5" s="2">
-        <f>0.5703</f>
-        <v>0.5703</v>
+        <v>0.8598</v>
       </c>
       <c r="P5" s="2">
-        <f>0.6603</f>
-        <v>0.6603</v>
+        <v>0.8734</v>
       </c>
       <c r="Q5" s="2">
-        <f>0.6517</f>
-        <v>0.6517</v>
+        <v>0.8746</v>
       </c>
     </row>
     <row r="6">
@@ -1717,16 +1693,16 @@
         <v>0.432</v>
       </c>
       <c r="N6" s="2">
-        <v>0.5724</v>
+        <v>0.7703</v>
       </c>
       <c r="O6" s="2">
-        <v>0.5237</v>
+        <v>0.7671</v>
       </c>
       <c r="P6" s="2">
-        <v>0.5039</v>
+        <v>0.8327</v>
       </c>
       <c r="Q6" s="2">
-        <v>0.4221</v>
+        <v>0.8322</v>
       </c>
     </row>
     <row r="7">
@@ -1770,20 +1746,16 @@
         <v>0.3979</v>
       </c>
       <c r="N7" s="2">
-        <f>0.5253</f>
-        <v>0.5253</v>
+        <v>0.6725</v>
       </c>
       <c r="O7" s="2">
-        <f>0.4403</f>
-        <v>0.4403</v>
+        <v>0.6458</v>
       </c>
       <c r="P7" s="2">
-        <f>0.4516</f>
-        <v>0.4516</v>
+        <v>0.7648</v>
       </c>
       <c r="Q7" s="2">
-        <f>0.3353</f>
-        <v>0.3353</v>
+        <v>0.7496</v>
       </c>
     </row>
   </sheetData>
@@ -1947,16 +1919,16 @@
         <v>0.5016</v>
       </c>
       <c r="N4" s="2">
-        <v>0.8853</v>
+        <v>0.8381</v>
       </c>
       <c r="O4" s="2">
-        <v>0.8856</v>
+        <v>0.8378</v>
       </c>
       <c r="P4" s="2">
-        <v>0.849</v>
+        <v>0.7672</v>
       </c>
       <c r="Q4" s="2">
-        <v>0.8474</v>
+        <v>0.7313</v>
       </c>
     </row>
     <row r="5">
@@ -2000,16 +1972,16 @@
         <v>0.5109</v>
       </c>
       <c r="N5" s="2">
-        <v>0.9077</v>
+        <v>0.8755</v>
       </c>
       <c r="O5" s="2">
-        <v>0.9089</v>
+        <v>0.8773</v>
       </c>
       <c r="P5" s="2">
-        <v>0.8741</v>
+        <v>0.8493</v>
       </c>
       <c r="Q5" s="2">
-        <v>0.873</v>
+        <v>0.844</v>
       </c>
     </row>
     <row r="6">
@@ -2053,16 +2025,16 @@
         <v>0.5326</v>
       </c>
       <c r="N6" s="2">
-        <v>0.8918</v>
+        <v>0.8941</v>
       </c>
       <c r="O6" s="2">
-        <v>0.893</v>
+        <v>0.8958</v>
       </c>
       <c r="P6" s="2">
-        <v>0.905</v>
+        <v>0.8843</v>
       </c>
       <c r="Q6" s="2">
-        <v>0.9062</v>
+        <v>0.8845</v>
       </c>
     </row>
     <row r="7">
@@ -2106,16 +2078,16 @@
         <v>0.5354</v>
       </c>
       <c r="N7" s="2">
-        <v>0.9101</v>
+        <v>0.8918</v>
       </c>
       <c r="O7" s="2">
-        <v>0.9105</v>
+        <v>0.893</v>
       </c>
       <c r="P7" s="2">
-        <v>0.905</v>
+        <v>0.8894</v>
       </c>
       <c r="Q7" s="2">
-        <v>0.9067</v>
+        <v>0.8903</v>
       </c>
     </row>
   </sheetData>
@@ -2279,16 +2251,16 @@
         <v>0.5424</v>
       </c>
       <c r="N4" s="2">
-        <v>0.9104</v>
+        <v>0.8918</v>
       </c>
       <c r="O4" s="2">
-        <v>0.9113</v>
+        <v>0.8927</v>
       </c>
       <c r="P4" s="2">
-        <v>0.9016</v>
+        <v>0.8924</v>
       </c>
       <c r="Q4" s="2">
-        <v>0.9032</v>
+        <v>0.8935</v>
       </c>
     </row>
     <row r="5">
@@ -2332,16 +2304,16 @@
         <v>0.5416</v>
       </c>
       <c r="N5" s="2">
-        <v>0.9009</v>
+        <v>0.887</v>
       </c>
       <c r="O5" s="2">
-        <v>0.9035</v>
+        <v>0.8875</v>
       </c>
       <c r="P5" s="2">
-        <v>0.9063</v>
+        <v>0.8911</v>
       </c>
       <c r="Q5" s="2">
-        <v>0.9075</v>
+        <v>0.892</v>
       </c>
     </row>
     <row r="6">
@@ -2385,16 +2357,16 @@
         <v>0.5376</v>
       </c>
       <c r="N6" s="2">
-        <v>0.8999</v>
+        <v>0.8765</v>
       </c>
       <c r="O6" s="2">
-        <v>0.9007</v>
+        <v>0.8762</v>
       </c>
       <c r="P6" s="2">
-        <v>0.8188</v>
+        <v>0.8863</v>
       </c>
       <c r="Q6" s="2">
-        <v>0.8138</v>
+        <v>0.8868</v>
       </c>
     </row>
     <row r="7">
@@ -2438,16 +2410,16 @@
         <v>0.5179</v>
       </c>
       <c r="N7" s="2">
-        <v>0.8853</v>
+        <v>0.8602</v>
       </c>
       <c r="O7" s="2">
-        <v>0.8867</v>
+        <v>0.8586</v>
       </c>
       <c r="P7" s="2">
-        <v>0.7957</v>
+        <v>0.8646</v>
       </c>
       <c r="Q7" s="2">
-        <v>0.7534</v>
+        <v>0.8639</v>
       </c>
     </row>
   </sheetData>
@@ -2611,20 +2583,16 @@
         <v>0.5319</v>
       </c>
       <c r="N4" s="2">
-        <f>0.9063</f>
-        <v>0.9063</v>
+        <v>0.8938</v>
       </c>
       <c r="O4" s="2">
-        <f>0.9083</f>
-        <v>0.9083</v>
+        <v>0.8949</v>
       </c>
       <c r="P4" s="2">
-        <f>0.9063</f>
-        <v>0.9063</v>
+        <v>0.8921</v>
       </c>
       <c r="Q4" s="2">
-        <f>0.9075</f>
-        <v>0.9075</v>
+        <v>0.8931</v>
       </c>
     </row>
     <row r="5">
@@ -2668,20 +2636,16 @@
         <v>0.5385</v>
       </c>
       <c r="N5" s="2">
-        <f>0.9013</f>
-        <v>0.9013</v>
+        <v>0.8935</v>
       </c>
       <c r="O5" s="2">
-        <f>0.903</f>
-        <v>0.903</v>
+        <v>0.8945</v>
       </c>
       <c r="P5" s="2">
-        <f>0.906</f>
-        <v>0.906</v>
+        <v>0.8931</v>
       </c>
       <c r="Q5" s="2">
-        <f>0.9082</f>
-        <v>0.9082</v>
+        <v>0.8942</v>
       </c>
     </row>
     <row r="6">
@@ -2725,20 +2689,16 @@
         <v>0.5421</v>
       </c>
       <c r="N6" s="2">
-        <f>0.9087</f>
-        <v>0.9087</v>
+        <v>0.8935</v>
       </c>
       <c r="O6" s="2">
-        <f>0.9094</f>
-        <v>0.9094</v>
+        <v>0.8945</v>
       </c>
       <c r="P6" s="2">
-        <f>0.8992</f>
-        <v>0.8992</v>
+        <v>0.8935</v>
       </c>
       <c r="Q6" s="2">
-        <f>0.9017</f>
-        <v>0.9017</v>
+        <v>0.8945</v>
       </c>
     </row>
     <row r="7">
@@ -2782,20 +2742,16 @@
         <v>0.5415</v>
       </c>
       <c r="N7" s="2">
-        <f>0.9006</f>
-        <v>0.9006</v>
+        <v>0.8935</v>
       </c>
       <c r="O7" s="2">
-        <f>0.9025</f>
-        <v>0.9025</v>
+        <v>0.8945</v>
       </c>
       <c r="P7" s="2">
-        <f>0.9141</f>
-        <v>0.9141</v>
+        <v>0.8935</v>
       </c>
       <c r="Q7" s="2">
-        <f>0.915</f>
-        <v>0.915</v>
+        <v>0.8945</v>
       </c>
     </row>
   </sheetData>

</xml_diff>